<commit_message>
chore: revert NIK import changes and keep only simple name and email insertion for calon afirmasi
</commit_message>
<xml_diff>
--- a/petugas afirmasi.xlsx
+++ b/petugas afirmasi.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="355">
   <si>
     <t>Nama</t>
   </si>
@@ -1076,16 +1076,10 @@
     <t>abtran843@gmail.com</t>
   </si>
   <si>
-    <t>NIK</t>
-  </si>
-  <si>
     <t>ananda Riza mahfudzi</t>
   </si>
   <si>
     <t>nandariza856@gmail.com</t>
-  </si>
-  <si>
-    <t>3321051106050003</t>
   </si>
 </sst>
 </file>
@@ -1534,7 +1528,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:E127"/>
+  <dimension ref="A1:D127"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="39.5703125" customWidth="true" style="0"/>
@@ -1543,7 +1537,7 @@
     <col min="4" max="4" width="24.5703125" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" customHeight="1" ht="15.75">
+    <row r="1" spans="1:4" customHeight="1" ht="15.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1556,11 +1550,8 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" customHeight="1" ht="15.75">
+    </row>
+    <row r="2" spans="1:4" customHeight="1" ht="15.75">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -1574,7 +1565,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:5" customHeight="1" ht="15.75">
+    <row r="3" spans="1:4" customHeight="1" ht="15.75">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1588,7 +1579,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:5" customHeight="1" ht="15.75">
+    <row r="4" spans="1:4" customHeight="1" ht="15.75">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -1602,7 +1593,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5" customHeight="1" ht="15.75">
+    <row r="5" spans="1:4" customHeight="1" ht="15.75">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -1616,7 +1607,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:5" customHeight="1" ht="15.75">
+    <row r="6" spans="1:4" customHeight="1" ht="15.75">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1630,7 +1621,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:5" customHeight="1" ht="15.75">
+    <row r="7" spans="1:4" customHeight="1" ht="15.75">
       <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
@@ -1644,7 +1635,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:5" customHeight="1" ht="15.75">
+    <row r="8" spans="1:4" customHeight="1" ht="15.75">
       <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
@@ -1658,7 +1649,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:5" customHeight="1" ht="15.75">
+    <row r="9" spans="1:4" customHeight="1" ht="15.75">
       <c r="A9" s="2" t="s">
         <v>22</v>
       </c>
@@ -1672,7 +1663,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:5" customHeight="1" ht="15.75">
+    <row r="10" spans="1:4" customHeight="1" ht="15.75">
       <c r="A10" s="2" t="s">
         <v>25</v>
       </c>
@@ -1686,7 +1677,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:5" customHeight="1" ht="15.75">
+    <row r="11" spans="1:4" customHeight="1" ht="15.75">
       <c r="A11" s="2" t="s">
         <v>27</v>
       </c>
@@ -1700,7 +1691,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:5" customHeight="1" ht="15.75">
+    <row r="12" spans="1:4" customHeight="1" ht="15.75">
       <c r="A12" s="2" t="s">
         <v>29</v>
       </c>
@@ -1714,7 +1705,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:5" customHeight="1" ht="15.75">
+    <row r="13" spans="1:4" customHeight="1" ht="15.75">
       <c r="A13" s="2" t="s">
         <v>32</v>
       </c>
@@ -1728,7 +1719,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:5" customHeight="1" ht="15.75">
+    <row r="14" spans="1:4" customHeight="1" ht="15.75">
       <c r="A14" s="2" t="s">
         <v>34</v>
       </c>
@@ -1742,7 +1733,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="15" spans="1:5" customHeight="1" ht="15.75">
+    <row r="15" spans="1:4" customHeight="1" ht="15.75">
       <c r="A15" s="2" t="s">
         <v>37</v>
       </c>
@@ -1756,7 +1747,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:5" customHeight="1" ht="15.75">
+    <row r="16" spans="1:4" customHeight="1" ht="15.75">
       <c r="A16" s="2" t="s">
         <v>39</v>
       </c>
@@ -1770,7 +1761,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:5" customHeight="1" ht="15.75">
+    <row r="17" spans="1:4" customHeight="1" ht="15.75">
       <c r="A17" s="2" t="s">
         <v>41</v>
       </c>
@@ -1784,7 +1775,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:5" customHeight="1" ht="15.75">
+    <row r="18" spans="1:4" customHeight="1" ht="15.75">
       <c r="A18" s="2" t="s">
         <v>44</v>
       </c>
@@ -1798,7 +1789,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:5" customHeight="1" ht="15.75">
+    <row r="19" spans="1:4" customHeight="1" ht="15.75">
       <c r="A19" s="2" t="s">
         <v>46</v>
       </c>
@@ -1812,7 +1803,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="20" spans="1:5" customHeight="1" ht="15.75">
+    <row r="20" spans="1:4" customHeight="1" ht="15.75">
       <c r="A20" s="2" t="s">
         <v>49</v>
       </c>
@@ -1826,7 +1817,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="21" spans="1:5" customHeight="1" ht="15.75">
+    <row r="21" spans="1:4" customHeight="1" ht="15.75">
       <c r="A21" s="2" t="s">
         <v>52</v>
       </c>
@@ -1840,7 +1831,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="22" spans="1:5" customHeight="1" ht="15.75">
+    <row r="22" spans="1:4" customHeight="1" ht="15.75">
       <c r="A22" s="2" t="s">
         <v>54</v>
       </c>
@@ -1854,7 +1845,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="23" spans="1:5" customHeight="1" ht="15.75">
+    <row r="23" spans="1:4" customHeight="1" ht="15.75">
       <c r="A23" s="2" t="s">
         <v>56</v>
       </c>
@@ -1868,7 +1859,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="24" spans="1:5" customHeight="1" ht="15.75">
+    <row r="24" spans="1:4" customHeight="1" ht="15.75">
       <c r="A24" s="2" t="s">
         <v>59</v>
       </c>
@@ -1882,7 +1873,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="1:5" customHeight="1" ht="15.75">
+    <row r="25" spans="1:4" customHeight="1" ht="15.75">
       <c r="A25" s="2" t="s">
         <v>61</v>
       </c>
@@ -1896,7 +1887,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="26" spans="1:5" customHeight="1" ht="15.75">
+    <row r="26" spans="1:4" customHeight="1" ht="15.75">
       <c r="A26" s="2" t="s">
         <v>63</v>
       </c>
@@ -1910,7 +1901,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:5" customHeight="1" ht="15.75">
+    <row r="27" spans="1:4" customHeight="1" ht="15.75">
       <c r="A27" s="1" t="s">
         <v>65</v>
       </c>
@@ -1924,7 +1915,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="28" spans="1:5" customHeight="1" ht="15.75">
+    <row r="28" spans="1:4" customHeight="1" ht="15.75">
       <c r="A28" s="2" t="s">
         <v>69</v>
       </c>
@@ -1938,7 +1929,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="29" spans="1:5" customHeight="1" ht="15.75">
+    <row r="29" spans="1:4" customHeight="1" ht="15.75">
       <c r="A29" s="2" t="s">
         <v>72</v>
       </c>
@@ -1952,7 +1943,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="30" spans="1:5" customHeight="1" ht="15.75">
+    <row r="30" spans="1:4" customHeight="1" ht="15.75">
       <c r="A30" s="2" t="s">
         <v>75</v>
       </c>
@@ -1966,7 +1957,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="31" spans="1:5" customHeight="1" ht="15.75">
+    <row r="31" spans="1:4" customHeight="1" ht="15.75">
       <c r="A31" s="2" t="s">
         <v>78</v>
       </c>
@@ -1980,7 +1971,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="32" spans="1:5" customHeight="1" ht="15.75">
+    <row r="32" spans="1:4" customHeight="1" ht="15.75">
       <c r="A32" s="2" t="s">
         <v>81</v>
       </c>
@@ -1994,7 +1985,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="33" spans="1:5" customHeight="1" ht="15.75">
+    <row r="33" spans="1:4" customHeight="1" ht="15.75">
       <c r="A33" s="2" t="s">
         <v>83</v>
       </c>
@@ -2008,7 +1999,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="34" spans="1:5" customHeight="1" ht="15.75">
+    <row r="34" spans="1:4" customHeight="1" ht="15.75">
       <c r="A34" s="1" t="s">
         <v>85</v>
       </c>
@@ -2022,7 +2013,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="35" spans="1:5" customHeight="1" ht="15.75">
+    <row r="35" spans="1:4" customHeight="1" ht="15.75">
       <c r="A35" s="1" t="s">
         <v>89</v>
       </c>
@@ -2036,7 +2027,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="36" spans="1:5" customHeight="1" ht="15.75">
+    <row r="36" spans="1:4" customHeight="1" ht="15.75">
       <c r="A36" s="1" t="s">
         <v>92</v>
       </c>
@@ -2050,7 +2041,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="37" spans="1:5" customHeight="1" ht="15.75">
+    <row r="37" spans="1:4" customHeight="1" ht="15.75">
       <c r="A37" s="1" t="s">
         <v>95</v>
       </c>
@@ -2064,7 +2055,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="38" spans="1:5" customHeight="1" ht="15.75">
+    <row r="38" spans="1:4" customHeight="1" ht="15.75">
       <c r="A38" s="1" t="s">
         <v>98</v>
       </c>
@@ -2078,7 +2069,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="39" spans="1:5" customHeight="1" ht="15.75">
+    <row r="39" spans="1:4" customHeight="1" ht="15.75">
       <c r="A39" s="1" t="s">
         <v>100</v>
       </c>
@@ -2092,7 +2083,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="40" spans="1:5" customHeight="1" ht="15.75">
+    <row r="40" spans="1:4" customHeight="1" ht="15.75">
       <c r="A40" s="1" t="s">
         <v>103</v>
       </c>
@@ -2106,7 +2097,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="41" spans="1:5" customHeight="1" ht="15.75">
+    <row r="41" spans="1:4" customHeight="1" ht="15.75">
       <c r="A41" s="1" t="s">
         <v>106</v>
       </c>
@@ -2120,7 +2111,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="42" spans="1:5" customHeight="1" ht="15.75">
+    <row r="42" spans="1:4" customHeight="1" ht="15.75">
       <c r="A42" s="2" t="s">
         <v>109</v>
       </c>
@@ -2134,7 +2125,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="43" spans="1:5" customHeight="1" ht="15.75">
+    <row r="43" spans="1:4" customHeight="1" ht="15.75">
       <c r="A43" s="2" t="s">
         <v>112</v>
       </c>
@@ -2148,7 +2139,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="44" spans="1:5" customHeight="1" ht="15.75">
+    <row r="44" spans="1:4" customHeight="1" ht="15.75">
       <c r="A44" s="2" t="s">
         <v>114</v>
       </c>
@@ -2162,7 +2153,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="45" spans="1:5" customHeight="1" ht="15.75">
+    <row r="45" spans="1:4" customHeight="1" ht="15.75">
       <c r="A45" s="1" t="s">
         <v>117</v>
       </c>
@@ -2176,7 +2167,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="46" spans="1:5" customHeight="1" ht="15.75">
+    <row r="46" spans="1:4" customHeight="1" ht="15.75">
       <c r="A46" s="1" t="s">
         <v>121</v>
       </c>
@@ -2190,7 +2181,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="47" spans="1:5" customHeight="1" ht="15.75">
+    <row r="47" spans="1:4" customHeight="1" ht="15.75">
       <c r="A47" s="1" t="s">
         <v>124</v>
       </c>
@@ -2204,7 +2195,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="48" spans="1:5" customHeight="1" ht="15.75">
+    <row r="48" spans="1:4" customHeight="1" ht="15.75">
       <c r="A48" s="1" t="s">
         <v>128</v>
       </c>
@@ -2218,7 +2209,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="49" spans="1:5" customHeight="1" ht="15.75">
+    <row r="49" spans="1:4" customHeight="1" ht="15.75">
       <c r="A49" s="1" t="s">
         <v>130</v>
       </c>
@@ -2232,7 +2223,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="50" spans="1:5" customHeight="1" ht="15.75">
+    <row r="50" spans="1:4" customHeight="1" ht="15.75">
       <c r="A50" s="1" t="s">
         <v>133</v>
       </c>
@@ -2246,7 +2237,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="51" spans="1:5" customHeight="1" ht="15.75">
+    <row r="51" spans="1:4" customHeight="1" ht="15.75">
       <c r="A51" s="1" t="s">
         <v>136</v>
       </c>
@@ -2260,7 +2251,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="52" spans="1:5" customHeight="1" ht="15.75">
+    <row r="52" spans="1:4" customHeight="1" ht="15.75">
       <c r="A52" s="1" t="s">
         <v>139</v>
       </c>
@@ -2274,7 +2265,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="53" spans="1:5" customHeight="1" ht="15.75">
+    <row r="53" spans="1:4" customHeight="1" ht="15.75">
       <c r="A53" s="1" t="s">
         <v>141</v>
       </c>
@@ -2288,7 +2279,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="54" spans="1:5" customHeight="1" ht="15.75">
+    <row r="54" spans="1:4" customHeight="1" ht="15.75">
       <c r="A54" s="1" t="s">
         <v>144</v>
       </c>
@@ -2302,7 +2293,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="55" spans="1:5" customHeight="1" ht="15.75">
+    <row r="55" spans="1:4" customHeight="1" ht="15.75">
       <c r="A55" s="1" t="s">
         <v>147</v>
       </c>
@@ -2316,7 +2307,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="56" spans="1:5" customHeight="1" ht="15.75">
+    <row r="56" spans="1:4" customHeight="1" ht="15.75">
       <c r="A56" s="1" t="s">
         <v>150</v>
       </c>
@@ -2330,7 +2321,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="57" spans="1:5" customHeight="1" ht="15.75">
+    <row r="57" spans="1:4" customHeight="1" ht="15.75">
       <c r="A57" s="1" t="s">
         <v>152</v>
       </c>
@@ -2344,7 +2335,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="58" spans="1:5" customHeight="1" ht="15.75">
+    <row r="58" spans="1:4" customHeight="1" ht="15.75">
       <c r="A58" s="1" t="s">
         <v>155</v>
       </c>
@@ -2358,7 +2349,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="59" spans="1:5" customHeight="1" ht="15.75">
+    <row r="59" spans="1:4" customHeight="1" ht="15.75">
       <c r="A59" s="1" t="s">
         <v>157</v>
       </c>
@@ -2372,7 +2363,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="60" spans="1:5" customHeight="1" ht="15.75">
+    <row r="60" spans="1:4" customHeight="1" ht="15.75">
       <c r="A60" s="1" t="s">
         <v>160</v>
       </c>
@@ -2386,7 +2377,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="61" spans="1:5" customHeight="1" ht="15.75">
+    <row r="61" spans="1:4" customHeight="1" ht="15.75">
       <c r="A61" s="1" t="s">
         <v>164</v>
       </c>
@@ -2400,7 +2391,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="62" spans="1:5" customHeight="1" ht="15.75">
+    <row r="62" spans="1:4" customHeight="1" ht="15.75">
       <c r="A62" s="1" t="s">
         <v>167</v>
       </c>
@@ -2414,7 +2405,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="63" spans="1:5" customHeight="1" ht="15.75">
+    <row r="63" spans="1:4" customHeight="1" ht="15.75">
       <c r="A63" s="1" t="s">
         <v>169</v>
       </c>
@@ -2428,7 +2419,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="64" spans="1:5" customHeight="1" ht="15.75">
+    <row r="64" spans="1:4" customHeight="1" ht="15.75">
       <c r="A64" s="1" t="s">
         <v>171</v>
       </c>
@@ -2442,7 +2433,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="65" spans="1:5" customHeight="1" ht="15.75">
+    <row r="65" spans="1:4" customHeight="1" ht="15.75">
       <c r="A65" s="1" t="s">
         <v>174</v>
       </c>
@@ -2456,7 +2447,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="66" spans="1:5" customHeight="1" ht="15.75">
+    <row r="66" spans="1:4" customHeight="1" ht="15.75">
       <c r="A66" s="1" t="s">
         <v>177</v>
       </c>
@@ -2470,7 +2461,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="67" spans="1:5" customHeight="1" ht="15.75">
+    <row r="67" spans="1:4" customHeight="1" ht="15.75">
       <c r="A67" s="1" t="s">
         <v>179</v>
       </c>
@@ -2484,7 +2475,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="68" spans="1:5" customHeight="1" ht="15.75">
+    <row r="68" spans="1:4" customHeight="1" ht="15.75">
       <c r="A68" s="1" t="s">
         <v>181</v>
       </c>
@@ -2498,7 +2489,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="69" spans="1:5" customHeight="1" ht="15.75">
+    <row r="69" spans="1:4" customHeight="1" ht="15.75">
       <c r="A69" s="1" t="s">
         <v>185</v>
       </c>
@@ -2512,7 +2503,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="70" spans="1:5" customHeight="1" ht="15.75">
+    <row r="70" spans="1:4" customHeight="1" ht="15.75">
       <c r="A70" s="1" t="s">
         <v>188</v>
       </c>
@@ -2526,7 +2517,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="71" spans="1:5" customHeight="1" ht="15.75">
+    <row r="71" spans="1:4" customHeight="1" ht="15.75">
       <c r="A71" s="1" t="s">
         <v>191</v>
       </c>
@@ -2540,7 +2531,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="72" spans="1:5" customHeight="1" ht="15.75">
+    <row r="72" spans="1:4" customHeight="1" ht="15.75">
       <c r="A72" s="2" t="s">
         <v>194</v>
       </c>
@@ -2554,7 +2545,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="73" spans="1:5" customHeight="1" ht="15.75">
+    <row r="73" spans="1:4" customHeight="1" ht="15.75">
       <c r="A73" s="2" t="s">
         <v>196</v>
       </c>
@@ -2568,7 +2559,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="74" spans="1:5" customHeight="1" ht="15.75">
+    <row r="74" spans="1:4" customHeight="1" ht="15.75">
       <c r="A74" s="1" t="s">
         <v>199</v>
       </c>
@@ -2582,7 +2573,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="75" spans="1:5" customHeight="1" ht="15.75">
+    <row r="75" spans="1:4" customHeight="1" ht="15.75">
       <c r="A75" s="1" t="s">
         <v>203</v>
       </c>
@@ -2596,7 +2587,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="76" spans="1:5" customHeight="1" ht="15.75">
+    <row r="76" spans="1:4" customHeight="1" ht="15.75">
       <c r="A76" s="2" t="s">
         <v>206</v>
       </c>
@@ -2610,7 +2601,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="77" spans="1:5" customHeight="1" ht="15.75">
+    <row r="77" spans="1:4" customHeight="1" ht="15.75">
       <c r="A77" s="2" t="s">
         <v>209</v>
       </c>
@@ -2624,7 +2615,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="78" spans="1:5" customHeight="1" ht="15.75">
+    <row r="78" spans="1:4" customHeight="1" ht="15.75">
       <c r="A78" s="2" t="s">
         <v>212</v>
       </c>
@@ -2638,7 +2629,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="79" spans="1:5" customHeight="1" ht="15.75">
+    <row r="79" spans="1:4" customHeight="1" ht="15.75">
       <c r="A79" s="2" t="s">
         <v>214</v>
       </c>
@@ -2652,7 +2643,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="80" spans="1:5" customHeight="1" ht="15.75">
+    <row r="80" spans="1:4" customHeight="1" ht="15.75">
       <c r="A80" s="2" t="s">
         <v>216</v>
       </c>
@@ -2666,7 +2657,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="81" spans="1:5" customHeight="1" ht="15.75">
+    <row r="81" spans="1:4" customHeight="1" ht="15.75">
       <c r="A81" s="2" t="s">
         <v>219</v>
       </c>
@@ -2680,7 +2671,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="82" spans="1:5" customHeight="1" ht="15.75">
+    <row r="82" spans="1:4" customHeight="1" ht="15.75">
       <c r="A82" s="1" t="s">
         <v>222</v>
       </c>
@@ -2694,7 +2685,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="83" spans="1:5" customHeight="1" ht="15.75">
+    <row r="83" spans="1:4" customHeight="1" ht="15.75">
       <c r="A83" s="1" t="s">
         <v>226</v>
       </c>
@@ -2708,7 +2699,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="84" spans="1:5" customHeight="1" ht="15.75">
+    <row r="84" spans="1:4" customHeight="1" ht="15.75">
       <c r="A84" s="1" t="s">
         <v>229</v>
       </c>
@@ -2722,7 +2713,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="85" spans="1:5" customHeight="1" ht="15.75">
+    <row r="85" spans="1:4" customHeight="1" ht="15.75">
       <c r="A85" s="1" t="s">
         <v>232</v>
       </c>
@@ -2736,7 +2727,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="86" spans="1:5" customHeight="1" ht="15.75">
+    <row r="86" spans="1:4" customHeight="1" ht="15.75">
       <c r="A86" s="1" t="s">
         <v>235</v>
       </c>
@@ -2750,7 +2741,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="87" spans="1:5" customHeight="1" ht="15.75">
+    <row r="87" spans="1:4" customHeight="1" ht="15.75">
       <c r="A87" s="1" t="s">
         <v>238</v>
       </c>
@@ -2764,7 +2755,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="88" spans="1:5" customHeight="1" ht="15.75">
+    <row r="88" spans="1:4" customHeight="1" ht="15.75">
       <c r="A88" s="1" t="s">
         <v>241</v>
       </c>
@@ -2778,7 +2769,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="89" spans="1:5" customHeight="1" ht="15.75">
+    <row r="89" spans="1:4" customHeight="1" ht="15.75">
       <c r="A89" s="1" t="s">
         <v>243</v>
       </c>
@@ -2792,7 +2783,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="90" spans="1:5" customHeight="1" ht="15.75">
+    <row r="90" spans="1:4" customHeight="1" ht="15.75">
       <c r="A90" s="2" t="s">
         <v>247</v>
       </c>
@@ -2806,7 +2797,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="91" spans="1:5" customHeight="1" ht="15.75">
+    <row r="91" spans="1:4" customHeight="1" ht="15.75">
       <c r="A91" s="2" t="s">
         <v>250</v>
       </c>
@@ -2820,7 +2811,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="92" spans="1:5" customHeight="1" ht="15.75">
+    <row r="92" spans="1:4" customHeight="1" ht="15.75">
       <c r="A92" s="2" t="s">
         <v>253</v>
       </c>
@@ -2834,7 +2825,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="93" spans="1:5" customHeight="1" ht="15.75">
+    <row r="93" spans="1:4" customHeight="1" ht="15.75">
       <c r="A93" s="2" t="s">
         <v>256</v>
       </c>
@@ -2848,7 +2839,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="94" spans="1:5" customHeight="1" ht="15.75">
+    <row r="94" spans="1:4" customHeight="1" ht="15.75">
       <c r="A94" s="2" t="s">
         <v>258</v>
       </c>
@@ -2862,7 +2853,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="95" spans="1:5" customHeight="1" ht="15.75">
+    <row r="95" spans="1:4" customHeight="1" ht="15.75">
       <c r="A95" s="2" t="s">
         <v>261</v>
       </c>
@@ -2876,7 +2867,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="96" spans="1:5" customHeight="1" ht="15.75">
+    <row r="96" spans="1:4" customHeight="1" ht="15.75">
       <c r="A96" s="2" t="s">
         <v>264</v>
       </c>
@@ -2890,7 +2881,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="97" spans="1:5" customHeight="1" ht="15.75">
+    <row r="97" spans="1:4" customHeight="1" ht="15.75">
       <c r="A97" s="1" t="s">
         <v>266</v>
       </c>
@@ -2904,7 +2895,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="98" spans="1:5" customHeight="1" ht="15.75">
+    <row r="98" spans="1:4" customHeight="1" ht="15.75">
       <c r="A98" s="1" t="s">
         <v>270</v>
       </c>
@@ -2918,7 +2909,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="99" spans="1:5" customHeight="1" ht="15.75">
+    <row r="99" spans="1:4" customHeight="1" ht="15.75">
       <c r="A99" s="1" t="s">
         <v>273</v>
       </c>
@@ -2932,7 +2923,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="100" spans="1:5" customHeight="1" ht="15.75">
+    <row r="100" spans="1:4" customHeight="1" ht="15.75">
       <c r="A100" s="1" t="s">
         <v>276</v>
       </c>
@@ -2946,7 +2937,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="101" spans="1:5" customHeight="1" ht="15.75">
+    <row r="101" spans="1:4" customHeight="1" ht="15.75">
       <c r="A101" s="1" t="s">
         <v>279</v>
       </c>
@@ -2960,7 +2951,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="102" spans="1:5" customHeight="1" ht="15.75">
+    <row r="102" spans="1:4" customHeight="1" ht="15.75">
       <c r="A102" s="1" t="s">
         <v>281</v>
       </c>
@@ -2974,7 +2965,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="103" spans="1:5" customHeight="1" ht="15.75">
+    <row r="103" spans="1:4" customHeight="1" ht="15.75">
       <c r="A103" s="1" t="s">
         <v>284</v>
       </c>
@@ -2988,7 +2979,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="104" spans="1:5" customHeight="1" ht="15.75">
+    <row r="104" spans="1:4" customHeight="1" ht="15.75">
       <c r="A104" s="1" t="s">
         <v>288</v>
       </c>
@@ -3002,7 +2993,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="105" spans="1:5" customHeight="1" ht="15.75">
+    <row r="105" spans="1:4" customHeight="1" ht="15.75">
       <c r="A105" s="1" t="s">
         <v>291</v>
       </c>
@@ -3016,7 +3007,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="106" spans="1:5" customHeight="1" ht="15.75">
+    <row r="106" spans="1:4" customHeight="1" ht="15.75">
       <c r="A106" s="1" t="s">
         <v>294</v>
       </c>
@@ -3030,7 +3021,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="107" spans="1:5" customHeight="1" ht="15.75">
+    <row r="107" spans="1:4" customHeight="1" ht="15.75">
       <c r="A107" s="1" t="s">
         <v>297</v>
       </c>
@@ -3044,7 +3035,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="108" spans="1:5" customHeight="1" ht="15.75">
+    <row r="108" spans="1:4" customHeight="1" ht="15.75">
       <c r="A108" s="1" t="s">
         <v>300</v>
       </c>
@@ -3058,7 +3049,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="109" spans="1:5" customHeight="1" ht="15.75">
+    <row r="109" spans="1:4" customHeight="1" ht="15.75">
       <c r="A109" s="2" t="s">
         <v>303</v>
       </c>
@@ -3072,7 +3063,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="110" spans="1:5" customHeight="1" ht="15.75">
+    <row r="110" spans="1:4" customHeight="1" ht="15.75">
       <c r="A110" s="2" t="s">
         <v>305</v>
       </c>
@@ -3086,7 +3077,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="111" spans="1:5" customHeight="1" ht="15.75">
+    <row r="111" spans="1:4" customHeight="1" ht="15.75">
       <c r="A111" s="2" t="s">
         <v>308</v>
       </c>
@@ -3100,7 +3091,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="112" spans="1:5" customHeight="1" ht="15.75">
+    <row r="112" spans="1:4" customHeight="1" ht="15.75">
       <c r="A112" s="2" t="s">
         <v>311</v>
       </c>
@@ -3114,7 +3105,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="113" spans="1:5" customHeight="1" ht="15.75">
+    <row r="113" spans="1:4" customHeight="1" ht="15.75">
       <c r="A113" s="2" t="s">
         <v>315</v>
       </c>
@@ -3128,7 +3119,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="114" spans="1:5" customHeight="1" ht="15.75">
+    <row r="114" spans="1:4" customHeight="1" ht="15.75">
       <c r="A114" s="2" t="s">
         <v>318</v>
       </c>
@@ -3142,7 +3133,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="115" spans="1:5" customHeight="1" ht="15.75">
+    <row r="115" spans="1:4" customHeight="1" ht="15.75">
       <c r="A115" s="3" t="s">
         <v>321</v>
       </c>
@@ -3156,7 +3147,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="116" spans="1:5" customHeight="1" ht="15.75">
+    <row r="116" spans="1:4" customHeight="1" ht="15.75">
       <c r="A116" s="2" t="s">
         <v>323</v>
       </c>
@@ -3170,7 +3161,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="117" spans="1:5" customHeight="1" ht="15.75">
+    <row r="117" spans="1:4" customHeight="1" ht="15.75">
       <c r="A117" s="1" t="s">
         <v>326</v>
       </c>
@@ -3184,7 +3175,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="118" spans="1:5" customHeight="1" ht="15.75">
+    <row r="118" spans="1:4" customHeight="1" ht="15.75">
       <c r="A118" s="1" t="s">
         <v>330</v>
       </c>
@@ -3198,7 +3189,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="119" spans="1:5" customHeight="1" ht="15.75">
+    <row r="119" spans="1:4" customHeight="1" ht="15.75">
       <c r="A119" s="1" t="s">
         <v>333</v>
       </c>
@@ -3212,7 +3203,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="120" spans="1:5" customHeight="1" ht="15.75">
+    <row r="120" spans="1:4" customHeight="1" ht="15.75">
       <c r="A120" s="1" t="s">
         <v>335</v>
       </c>
@@ -3226,7 +3217,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="121" spans="1:5" customHeight="1" ht="15.75">
+    <row r="121" spans="1:4" customHeight="1" ht="15.75">
       <c r="A121" s="1" t="s">
         <v>338</v>
       </c>
@@ -3240,7 +3231,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="122" spans="1:5" customHeight="1" ht="15.75">
+    <row r="122" spans="1:4" customHeight="1" ht="15.75">
       <c r="A122" s="1" t="s">
         <v>340</v>
       </c>
@@ -3254,7 +3245,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="123" spans="1:5" customHeight="1" ht="15.75">
+    <row r="123" spans="1:4" customHeight="1" ht="15.75">
       <c r="A123" s="1" t="s">
         <v>342</v>
       </c>
@@ -3268,7 +3259,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="124" spans="1:5" customHeight="1" ht="15.75">
+    <row r="124" spans="1:4" customHeight="1" ht="15.75">
       <c r="A124" s="4" t="s">
         <v>345</v>
       </c>
@@ -3282,7 +3273,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="125" spans="1:5" customHeight="1" ht="15.75">
+    <row r="125" spans="1:4" customHeight="1" ht="15.75">
       <c r="A125" s="5" t="s">
         <v>349</v>
       </c>
@@ -3290,7 +3281,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="126" spans="1:5" customHeight="1" ht="15.75">
+    <row r="126" spans="1:4" customHeight="1" ht="15.75">
       <c r="A126" s="5" t="s">
         <v>351</v>
       </c>
@@ -3298,18 +3289,15 @@
         <v>352</v>
       </c>
     </row>
-    <row r="127" spans="1:5">
+    <row r="127" spans="1:4">
       <c r="A127" t="s">
+        <v>353</v>
+      </c>
+      <c r="B127" t="s">
         <v>354</v>
-      </c>
-      <c r="B127" t="s">
-        <v>355</v>
       </c>
       <c r="C127"/>
       <c r="D127"/>
-      <c r="E127" t="s">
-        <v>356</v>
-      </c>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>

<commit_message>
feat: add Ghulam Za'imul Haq and ananda Riza mahfudzi to DB and petugas afirmasi spreadsheet
</commit_message>
<xml_diff>
--- a/petugas afirmasi.xlsx
+++ b/petugas afirmasi.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="357">
   <si>
     <t>Nama</t>
   </si>
@@ -1080,6 +1080,12 @@
   </si>
   <si>
     <t>nandariza856@gmail.com</t>
+  </si>
+  <si>
+    <t>Ghulam Za'imul Haq</t>
+  </si>
+  <si>
+    <t>ghulamzaim01@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -1528,7 +1534,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D127"/>
+  <dimension ref="A1:D128"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="39.5703125" customWidth="true" style="0"/>
@@ -3298,6 +3304,16 @@
       </c>
       <c r="C127"/>
       <c r="D127"/>
+    </row>
+    <row r="128" spans="1:4">
+      <c r="A128" t="s">
+        <v>355</v>
+      </c>
+      <c r="B128" t="s">
+        <v>356</v>
+      </c>
+      <c r="C128"/>
+      <c r="D128"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>

<commit_message>
feat: add Lailatus Sa'adah to DB and petugas afirmasi spreadsheet
</commit_message>
<xml_diff>
--- a/petugas afirmasi.xlsx
+++ b/petugas afirmasi.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="359">
   <si>
     <t>Nama</t>
   </si>
@@ -1086,6 +1086,12 @@
   </si>
   <si>
     <t>ghulamzaim01@gmail.com</t>
+  </si>
+  <si>
+    <t>Lailatus Sa'adah</t>
+  </si>
+  <si>
+    <t>lailatus95.2012@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -1534,7 +1540,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D128"/>
+  <dimension ref="A1:D129"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="39.5703125" customWidth="true" style="0"/>
@@ -3314,6 +3320,16 @@
       </c>
       <c r="C128"/>
       <c r="D128"/>
+    </row>
+    <row r="129" spans="1:4">
+      <c r="A129" t="s">
+        <v>357</v>
+      </c>
+      <c r="B129" t="s">
+        <v>358</v>
+      </c>
+      <c r="C129"/>
+      <c r="D129"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>

<commit_message>
feat: add 4 new calon afirmasi to DB and spreadsheet
</commit_message>
<xml_diff>
--- a/petugas afirmasi.xlsx
+++ b/petugas afirmasi.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="367">
   <si>
     <t>Nama</t>
   </si>
@@ -1092,6 +1092,30 @@
   </si>
   <si>
     <t>lailatus95.2012@gmail.com</t>
+  </si>
+  <si>
+    <t>Abdus salam</t>
+  </si>
+  <si>
+    <t>alvinsalam93@gmail.com</t>
+  </si>
+  <si>
+    <t>MOHAMAD HARIS WIYANTO</t>
+  </si>
+  <si>
+    <t>ariswedung32@gmail.com</t>
+  </si>
+  <si>
+    <t>herdi sofyan</t>
+  </si>
+  <si>
+    <t>Herdialdino160@gmail.com</t>
+  </si>
+  <si>
+    <t>Nailul Muna</t>
+  </si>
+  <si>
+    <t>nailulmuna48@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -1540,7 +1564,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D129"/>
+  <dimension ref="A1:D133"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="39.5703125" customWidth="true" style="0"/>
@@ -3330,6 +3354,46 @@
       </c>
       <c r="C129"/>
       <c r="D129"/>
+    </row>
+    <row r="130" spans="1:4">
+      <c r="A130" t="s">
+        <v>359</v>
+      </c>
+      <c r="B130" t="s">
+        <v>360</v>
+      </c>
+      <c r="C130"/>
+      <c r="D130"/>
+    </row>
+    <row r="131" spans="1:4">
+      <c r="A131" t="s">
+        <v>361</v>
+      </c>
+      <c r="B131" t="s">
+        <v>362</v>
+      </c>
+      <c r="C131"/>
+      <c r="D131"/>
+    </row>
+    <row r="132" spans="1:4">
+      <c r="A132" t="s">
+        <v>363</v>
+      </c>
+      <c r="B132" t="s">
+        <v>364</v>
+      </c>
+      <c r="C132"/>
+      <c r="D132"/>
+    </row>
+    <row r="133" spans="1:4">
+      <c r="A133" t="s">
+        <v>365</v>
+      </c>
+      <c r="B133" t="s">
+        <v>366</v>
+      </c>
+      <c r="C133"/>
+      <c r="D133"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>

<commit_message>
feat: add Choirul fasikhin to DB and spreadsheet
</commit_message>
<xml_diff>
--- a/petugas afirmasi.xlsx
+++ b/petugas afirmasi.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="369">
   <si>
     <t>Nama</t>
   </si>
@@ -1116,6 +1116,12 @@
   </si>
   <si>
     <t>nailulmuna48@gmail.com</t>
+  </si>
+  <si>
+    <t>Choirul fasikhin</t>
+  </si>
+  <si>
+    <t>choirul.akin@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -1564,7 +1570,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D133"/>
+  <dimension ref="A1:D134"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="39.5703125" customWidth="true" style="0"/>
@@ -3394,6 +3400,16 @@
       </c>
       <c r="C133"/>
       <c r="D133"/>
+    </row>
+    <row r="134" spans="1:4">
+      <c r="A134" t="s">
+        <v>367</v>
+      </c>
+      <c r="B134" t="s">
+        <v>368</v>
+      </c>
+      <c r="C134"/>
+      <c r="D134"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>

<commit_message>
feat: add Mohamad Khoirul Huda to DB and spreadsheet
</commit_message>
<xml_diff>
--- a/petugas afirmasi.xlsx
+++ b/petugas afirmasi.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="371">
   <si>
     <t>Nama</t>
   </si>
@@ -1122,6 +1122,12 @@
   </si>
   <si>
     <t>choirul.akin@gmail.com</t>
+  </si>
+  <si>
+    <t>Mohamad Khoirul Huda</t>
+  </si>
+  <si>
+    <t>mkhoirulhuda2003@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -1570,7 +1576,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D134"/>
+  <dimension ref="A1:D135"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="39.5703125" customWidth="true" style="0"/>
@@ -3410,6 +3416,16 @@
       </c>
       <c r="C134"/>
       <c r="D134"/>
+    </row>
+    <row r="135" spans="1:4">
+      <c r="A135" t="s">
+        <v>369</v>
+      </c>
+      <c r="B135" t="s">
+        <v>370</v>
+      </c>
+      <c r="C135"/>
+      <c r="D135"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>

<commit_message>
feat: add sri lestari to DB and spreadsheet
</commit_message>
<xml_diff>
--- a/petugas afirmasi.xlsx
+++ b/petugas afirmasi.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="373">
   <si>
     <t>Nama</t>
   </si>
@@ -1128,6 +1128,12 @@
   </si>
   <si>
     <t>mkhoirulhuda2003@gmail.com</t>
+  </si>
+  <si>
+    <t>sri lestari</t>
+  </si>
+  <si>
+    <t>lestarimanis321@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -1576,7 +1582,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D135"/>
+  <dimension ref="A1:D136"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="39.5703125" customWidth="true" style="0"/>
@@ -3426,6 +3432,16 @@
       </c>
       <c r="C135"/>
       <c r="D135"/>
+    </row>
+    <row r="136" spans="1:4">
+      <c r="A136" t="s">
+        <v>371</v>
+      </c>
+      <c r="B136" t="s">
+        <v>372</v>
+      </c>
+      <c r="C136"/>
+      <c r="D136"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>

<commit_message>
feat: add Suyanti and muhammad dany Ariyanto to DB and spreadsheet
</commit_message>
<xml_diff>
--- a/petugas afirmasi.xlsx
+++ b/petugas afirmasi.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="377">
   <si>
     <t>Nama</t>
   </si>
@@ -1134,6 +1134,18 @@
   </si>
   <si>
     <t>lestarimanis321@gmail.com</t>
+  </si>
+  <si>
+    <t>Suyanti</t>
+  </si>
+  <si>
+    <t>suyanyanti81@gmail.com</t>
+  </si>
+  <si>
+    <t>muhammad dany Ariyanto</t>
+  </si>
+  <si>
+    <t>mdanyrizqianto@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -1582,7 +1594,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D136"/>
+  <dimension ref="A1:D138"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="39.5703125" customWidth="true" style="0"/>
@@ -3442,6 +3454,26 @@
       </c>
       <c r="C136"/>
       <c r="D136"/>
+    </row>
+    <row r="137" spans="1:4">
+      <c r="A137" t="s">
+        <v>373</v>
+      </c>
+      <c r="B137" t="s">
+        <v>374</v>
+      </c>
+      <c r="C137"/>
+      <c r="D137"/>
+    </row>
+    <row r="138" spans="1:4">
+      <c r="A138" t="s">
+        <v>375</v>
+      </c>
+      <c r="B138" t="s">
+        <v>376</v>
+      </c>
+      <c r="C138"/>
+      <c r="D138"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>

<commit_message>
feat: add Itsni Faiq, Dwi Selvaa, and Meylla to DB and spreadsheet
</commit_message>
<xml_diff>
--- a/petugas afirmasi.xlsx
+++ b/petugas afirmasi.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="383">
   <si>
     <t>Nama</t>
   </si>
@@ -1146,6 +1146,24 @@
   </si>
   <si>
     <t>mdanyrizqianto@gmail.com</t>
+  </si>
+  <si>
+    <t>Itsni Faiq</t>
+  </si>
+  <si>
+    <t>ibrahimovaic@gmail.com</t>
+  </si>
+  <si>
+    <t>Dwi Selvaa Maulidenna</t>
+  </si>
+  <si>
+    <t>dmaulidenna@gmail.com</t>
+  </si>
+  <si>
+    <t>Meylla erviana putri</t>
+  </si>
+  <si>
+    <t>meyllap76@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -1594,7 +1612,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D138"/>
+  <dimension ref="A1:D141"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="39.5703125" customWidth="true" style="0"/>
@@ -3474,6 +3492,36 @@
       </c>
       <c r="C138"/>
       <c r="D138"/>
+    </row>
+    <row r="139" spans="1:4">
+      <c r="A139" t="s">
+        <v>377</v>
+      </c>
+      <c r="B139" t="s">
+        <v>378</v>
+      </c>
+      <c r="C139"/>
+      <c r="D139"/>
+    </row>
+    <row r="140" spans="1:4">
+      <c r="A140" t="s">
+        <v>379</v>
+      </c>
+      <c r="B140" t="s">
+        <v>380</v>
+      </c>
+      <c r="C140"/>
+      <c r="D140"/>
+    </row>
+    <row r="141" spans="1:4">
+      <c r="A141" t="s">
+        <v>381</v>
+      </c>
+      <c r="B141" t="s">
+        <v>382</v>
+      </c>
+      <c r="C141"/>
+      <c r="D141"/>
     </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>

</xml_diff>